<commit_message>
Update action ladder reference with Marc's final owner decisions
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MTG_Action_Ladder_Reference_v2.xlsx
+++ b/docs/MTG_Action_Ladder_Reference_v2.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Tyler/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D614E7C2-D124-184C-B09A-9EC9216DF02E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93F505FB-6B4E-0149-A6B2-B3E406FBAF91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51200" yWindow="7800" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Action Ladder Reference" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Ladder Reference'!$A$1:$F$113</definedName>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="198">
   <si>
     <t>Sub-Path</t>
   </si>
@@ -667,7 +668,7 @@
       <name val="Inter"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -699,6 +700,12 @@
         <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -727,7 +734,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -745,6 +752,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1721,8 +1731,8 @@
       <c r="D37" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="E37" s="4" t="s">
-        <v>13</v>
+      <c r="E37" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>14</v>
@@ -2147,22 +2157,22 @@
       </c>
     </row>
     <row r="61" spans="1:6" ht="28">
-      <c r="A61" s="4" t="s">
+      <c r="A61" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B61" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C61" s="4" t="s">
+      <c r="C61" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="D61" s="4" t="s">
+      <c r="D61" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E61" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F61" s="4" t="s">
+      <c r="E61" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F61" s="7" t="s">
         <v>14</v>
       </c>
     </row>
@@ -2419,22 +2429,22 @@
       <c r="F75" s="2"/>
     </row>
     <row r="76" spans="1:6" ht="28">
-      <c r="A76" s="3" t="s">
+      <c r="A76" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B76" s="3" t="s">
+      <c r="B76" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C76" s="3" t="s">
+      <c r="C76" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="D76" s="3" t="s">
+      <c r="D76" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="E76" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F76" s="3" t="s">
+      <c r="E76" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F76" s="7" t="s">
         <v>14</v>
       </c>
     </row>
@@ -2519,22 +2529,22 @@
       </c>
     </row>
     <row r="81" spans="1:6" ht="28">
-      <c r="A81" s="4" t="s">
+      <c r="A81" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B81" s="4" t="s">
+      <c r="B81" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C81" s="4" t="s">
+      <c r="C81" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="D81" s="4" t="s">
+      <c r="D81" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="E81" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F81" s="4" t="s">
+      <c r="E81" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F81" s="7" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2645,22 +2655,22 @@
       </c>
     </row>
     <row r="88" spans="1:6" ht="28">
-      <c r="A88" s="3" t="s">
+      <c r="A88" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="B88" s="3" t="s">
+      <c r="B88" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C88" s="3" t="s">
+      <c r="C88" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="D88" s="3" t="s">
+      <c r="D88" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="E88" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F88" s="3" t="s">
+      <c r="E88" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F88" s="7" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2791,22 +2801,22 @@
       </c>
     </row>
     <row r="96" spans="1:6" ht="28">
-      <c r="A96" s="3" t="s">
+      <c r="A96" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="B96" s="3" t="s">
+      <c r="B96" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C96" s="3" t="s">
+      <c r="C96" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="D96" s="3" t="s">
+      <c r="D96" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="E96" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F96" s="3" t="s">
+      <c r="E96" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F96" s="7" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2857,22 +2867,22 @@
       <c r="F99" s="2"/>
     </row>
     <row r="100" spans="1:6" ht="28">
-      <c r="A100" s="3" t="s">
+      <c r="A100" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B100" s="3" t="s">
+      <c r="B100" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C100" s="3" t="s">
+      <c r="C100" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="D100" s="3" t="s">
+      <c r="D100" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="E100" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F100" s="3" t="s">
+      <c r="E100" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F100" s="7" t="s">
         <v>14</v>
       </c>
     </row>
@@ -2897,22 +2907,22 @@
       </c>
     </row>
     <row r="102" spans="1:6" ht="28">
-      <c r="A102" s="3" t="s">
+      <c r="A102" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B102" s="3" t="s">
+      <c r="B102" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C102" s="3" t="s">
+      <c r="C102" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="D102" s="3" t="s">
+      <c r="D102" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="E102" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F102" s="3" t="s">
+      <c r="E102" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F102" s="7" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2937,22 +2947,22 @@
       </c>
     </row>
     <row r="104" spans="1:6" ht="28">
-      <c r="A104" s="3" t="s">
+      <c r="A104" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B104" s="3" t="s">
+      <c r="B104" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C104" s="3" t="s">
+      <c r="C104" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="D104" s="3" t="s">
+      <c r="D104" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="E104" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F104" s="3" t="s">
+      <c r="E104" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F104" s="7" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3125,11 +3135,6 @@
   </sheetData>
   <autoFilter ref="A1:F113" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="14">
-    <mergeCell ref="A98:F98"/>
-    <mergeCell ref="A66:F66"/>
-    <mergeCell ref="A106:F106"/>
-    <mergeCell ref="A58:F58"/>
-    <mergeCell ref="A74:F74"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A42:F42"/>
@@ -3139,7 +3144,182 @@
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A98:F98"/>
+    <mergeCell ref="A66:F66"/>
+    <mergeCell ref="A106:F106"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A74:F74"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{361149D2-D9D0-C146-8A57-2F5035CC9353}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6" ht="98">
+      <c r="A1" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="84">
+      <c r="A2" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="98">
+      <c r="A3" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="98">
+      <c r="A4" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="98">
+      <c r="A5" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="84">
+      <c r="A6" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="112">
+      <c r="A7" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="98">
+      <c r="A8" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>